<commit_message>
feat: implement group by validator
</commit_message>
<xml_diff>
--- a/config/validation_config.xlsx
+++ b/config/validation_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\dw-data-validator\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DAA352E8-E2B0-4E57-9A0A-E0E53103ED20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E10546E8-F88C-4C5D-8C4A-B5B2F0302085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2309F37C-6F46-4C4C-A72F-FCDA6EABE24E}"/>
+    <workbookView xWindow="8085" yWindow="3600" windowWidth="21600" windowHeight="11295" xr2:uid="{2309F37C-6F46-4C4C-A72F-FCDA6EABE24E}"/>
   </bookViews>
   <sheets>
     <sheet name="ValidationConfig" sheetId="1" r:id="rId1"/>
@@ -75,9 +75,6 @@
     <t>sale_id</t>
   </si>
   <si>
-    <t>sale_dt</t>
-  </si>
-  <si>
     <t>qty,sale_amt</t>
   </si>
   <si>
@@ -94,6 +91,10 @@
   </si>
   <si>
     <t>비교 대상 컬럼(','로 구분)</t>
+  </si>
+  <si>
+    <t>store_cd</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -148,15 +149,12 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -495,13 +493,13 @@
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.875" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.25" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.125" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.625" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.875" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.25" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.25" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -528,26 +526,26 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" t="s">
         <v>12</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -561,33 +559,32 @@
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="9" style="2"/>
+    <col min="1" max="1" width="21.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>16</v>
+      <c r="B2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>17</v>
+      <c r="B3" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add validation execution time measurement
</commit_message>
<xml_diff>
--- a/config/validation_config.xlsx
+++ b/config/validation_config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\dw-data-validator\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66DEEEC7-D903-46D8-A72F-2BBB39F87601}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{031C114B-B53B-4FBA-A185-F7380E2B4947}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3705" yWindow="2700" windowWidth="21600" windowHeight="11295" xr2:uid="{2309F37C-6F46-4C4C-A72F-FCDA6EABE24E}"/>
+    <workbookView xWindow="9945" yWindow="6015" windowWidth="17190" windowHeight="13230" xr2:uid="{2309F37C-6F46-4C4C-A72F-FCDA6EABE24E}"/>
   </bookViews>
   <sheets>
     <sheet name="ValidationConfig" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="33">
   <si>
     <t>VALIDATION_NAME</t>
   </si>
@@ -63,37 +63,100 @@
     <t>USE_YN</t>
   </si>
   <si>
-    <t>Sales Validation</t>
-  </si>
-  <si>
-    <t>valid.ods_sales</t>
-  </si>
-  <si>
-    <t>valid.fact_sales</t>
-  </si>
-  <si>
-    <t>sale_id</t>
-  </si>
-  <si>
-    <t>qty,sale_amt</t>
+    <t>컬럼</t>
+  </si>
+  <si>
+    <t>설명</t>
+  </si>
+  <si>
+    <t>PK 컬럼명(','로 구분)</t>
+  </si>
+  <si>
+    <t>비교 대상 컬럼(','로 구분)</t>
+  </si>
+  <si>
+    <t>ods.krx_sto_knx_isu_base_info</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>isu_cd,mkt_tp_nm</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>parval</t>
+  </si>
+  <si>
+    <t>list_dd</t>
+  </si>
+  <si>
+    <t>N</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ods.krx_sto_ksq_isu_base_info</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>Y</t>
-  </si>
-  <si>
-    <t>컬럼</t>
-  </si>
-  <si>
-    <t>설명</t>
-  </si>
-  <si>
-    <t>PK 컬럼명(','로 구분)</t>
-  </si>
-  <si>
-    <t>비교 대상 컬럼(','로 구분)</t>
-  </si>
-  <si>
-    <t>store_cd</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Validation Time110</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Validation Time1820</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ods.massive_tickers_info</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Validation Time12308</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ticker</t>
+  </si>
+  <si>
+    <t>ods.krx_idx_kospi_dd_trd</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Validation Time72353</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>bas_dd,idx_clss,idx_nm</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>idx_clss</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>cmpprevdd_idx</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ods.krx_esg_sri_bond_info</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Validation Time3353153</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>bas_dd,isur_nm,isu_cd</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>bas_dd</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>isu_amt,list_amt</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -490,7 +553,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CC4FBC8-FC71-4C2B-904F-E4471707E210}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.875" bestFit="1" customWidth="1"/>
@@ -527,25 +590,111 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" t="s">
+        <v>27</v>
+      </c>
+      <c r="G5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" t="s">
+        <v>32</v>
+      </c>
+      <c r="G6" t="s">
         <v>17</v>
-      </c>
-      <c r="F2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -565,10 +714,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -576,7 +725,7 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -584,7 +733,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>